<commit_message>
checkpoint - breaking code up
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/facilities.xlsx
+++ b/reconcile/storage/output/facilities.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2944,32 +2944,32 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>h tec systems</t>
+          <t>ilika</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Hampshire</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>{'east': 10.32527718680763, 'south': 53.39508508510774, 'north': 53.73943730358849, 'west': 9.730130859481674, 'accuracyLevel': 10}</t>
+          <t>{'east': -1.449094865107286, 'south': 50.980418567607344, 'north': 51.008842561168144, 'west': -1.508401206810452, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>hydrogen</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -2982,22 +2982,22 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ilika</t>
+          <t>aesc</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Hampshire</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>{'east': -1.449094865107286, 'south': 50.980418567607344, 'north': 51.008842561168144, 'west': -1.508401206810452, 'accuracyLevel': 10}</t>
+          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>aesc</t>
+          <t>automotive cell company</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.844677657505151, 'south': 50.50016935124857, 'north': 50.51815664875143, 'west': 2.816388342494849, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['cell' 'module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>automotive cell company</t>
+          <t>automotive energy supply company</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>{'east': 2.844677657505151, 'south': 50.50016935124857, 'north': 50.51815664875143, 'west': 2.816388342494849, 'accuracyLevel': 2}</t>
+          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack' nan]</t>
+          <t>['cell' 'module_pack']</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>automotive energy supply company</t>
+          <t>byd</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3111,17 +3111,17 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.121182808680378, 'south': 49.40413017562429, 'north': 49.41312382437572, 'west': 2.107359191319622, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>byd</t>
+          <t>eramet suez</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3149,17 +3149,17 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>{'east': 2.121182808680378, 'south': 49.40413017562429, 'north': 49.41312382437572, 'west': 2.107359191319622, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>eramet suez</t>
+          <t>li cycle</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.9282400719596318, 'south': 50.431512720797635, 'north': 50.461341279202365, 'west': 2.8813839280403686, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>li cycle</t>
+          <t>prologium</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>{'east': 2.9282400719596318, 'south': 50.431512720797635, 'north': 50.461341279202365, 'west': 2.8813839280403686, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>prologium</t>
+          <t>renault</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
+          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>[nan 'cell']</t>
         </is>
       </c>
     </row>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>[nan 'cell']</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>renault group</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3344,12 +3344,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>renault group</t>
+          <t>renault minth</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>{'east': 3.122708534247327, 'south': 50.34297071284946, 'north': 50.398411287150545, 'west': 3.035735465752673, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.5958222612039354, 'south': 50.46193117562429, 'north': 50.470924824375714, 'west': 2.581691738796065, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>renault minth</t>
+          <t>saft</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>{'east': 2.5958222612039354, 'south': 50.46193117562429, 'north': 50.470924824375714, 'west': 2.581691738796065, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.844677657505151, 'south': 50.50016935124857, 'north': 50.51815664875143, 'west': 2.816388342494849, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>saft</t>
+          <t>toyota motor europe</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3453,17 +3453,17 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>{'east': 2.844677657505151, 'south': 50.50016935124857, 'north': 50.51815664875143, 'west': 2.816388342494849, 'accuracyLevel': 2}</t>
+          <t>{'east': 3.5679556995225914, 'south': 50.33173888518208, 'north': 50.38644511481792, 'west': 3.482156300477409, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>toyota motor europe</t>
+          <t>verkor</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3491,17 +3491,17 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>{'east': 3.5679556995225914, 'south': 50.33173888518208, 'north': 50.38644511481792, 'west': 3.482156300477409, 'accuracyLevel': 2}</t>
+          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -3514,22 +3514,22 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>verkor</t>
+          <t>akasol</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Hesse</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>{'east': 2.431777535628651, 'south': 50.99985923656883, 'north': 51.068940763431165, 'west': 2.3218424643713487, 'accuracyLevel': 2}</t>
+          <t>{'east': 8.686620210377718, 'south': 49.84474495759695, 'north': 49.899698335693174, 'west': 8.615127588265333, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -3552,22 +3552,22 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>akasol</t>
+          <t>glencore britishvolt</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Hesse</t>
+          <t>Kent</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>{'east': 8.686620210377718, 'south': 49.84474495759695, 'north': 49.899698335693174, 'west': 8.615127588265333, 'accuracyLevel': 10}</t>
+          <t>{'east': 0.3613610796854584, 'south': 51.417670417209834, 'north': 51.46163963815849, 'west': 0.31142776951638473, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>['module_pack' nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>glencore britishvolt</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3600,22 +3600,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Kent</t>
+          <t>Knowsley</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>{'east': 0.3613610796854584, 'south': 51.417670417209834, 'north': 51.46163963815849, 'west': 0.31142776951638473, 'accuracyLevel': 10}</t>
+          <t>{'east': -2.7848325756101486, 'south': 53.346631287550544, 'north': 53.3820389197578, 'west': -2.8562320000766497, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -3628,22 +3628,22 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>byd</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Knowsley</t>
+          <t>Komárom-Esztergom</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>{'east': -2.7848325756101486, 'south': 53.346631287550544, 'north': 53.3820389197578, 'west': -2.8562320000766497, 'accuracyLevel': 10}</t>
+          <t>{'east': 18.14503799430183, 'south': 47.72576787408204, 'north': 47.76060012591796, 'west': 18.093222005698166, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>byd</t>
+          <t>huayou cobalt</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>{'east': 18.14503799430183, 'south': 47.72576787408204, 'north': 47.76060012591796, 'west': 18.093222005698166, 'accuracyLevel': 2}</t>
+          <t>{'east': 18.02626000679121, 'south': 47.70225879501302, 'north': 47.722369204986975, 'west': 17.99636599320879, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>huayou cobalt</t>
+          <t>sk innovation</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>{'east': 18.02626000679121, 'south': 47.70225879501302, 'north': 47.722369204986975, 'west': 17.99636599320879, 'accuracyLevel': 2}</t>
+          <t>{'east': 18.14503799430183, 'south': 47.72576787408204, 'north': 47.76060012591796, 'west': 18.093222005698166, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -3742,32 +3742,32 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>sk innovation</t>
+          <t>volvo cars</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Komárom-Esztergom</t>
+          <t>Košice Region</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>{'east': 18.14503799430183, 'south': 47.72576787408204, 'north': 47.76060012591796, 'west': 18.093222005698166, 'accuracyLevel': 2}</t>
+          <t>{'east': 21.352141564262467, 'south': 48.651961553575575, 'north': 48.775930446424425, 'west': 21.164026435737533, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>volvo cars</t>
+          <t>zhi dou</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3818,32 +3818,32 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>zhi dou</t>
+          <t>easpring finland new materials oy</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Košice Region</t>
+          <t>Kymenlaakso</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>{'east': 21.352141564262467, 'south': 48.651961553575575, 'north': 48.775930446424425, 'west': 21.164026435737533, 'accuracyLevel': 2}</t>
+          <t>{'east': 27.007073004073145, 'south': 60.43623438503798, 'north': 60.49656561496202, 'west': 26.884566995926857, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>easpring finland new materials oy</t>
+          <t>finnish minerals beijing easpring</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>finnish minerals beijing easpring</t>
+          <t>finnish minerals group</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -3932,32 +3932,32 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>finnish minerals group</t>
+          <t>baywa re</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Kymenlaakso</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>{'east': 27.007073004073145, 'south': 60.43623438503798, 'north': 60.49656561496202, 'west': 26.884566995926857, 'accuracyLevel': 2}</t>
+          <t>{'east': 11.768207246122227, 'south': 42.237743552077085, 'north': 42.25745641692802, 'west': 11.740996804661673, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['deployment']</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>baywa re</t>
+          <t>lotus</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Leicestershire</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>{'east': 11.768207246122227, 'south': 42.237743552077085, 'north': 42.25745641692802, 'west': 11.740996804661673, 'accuracyLevel': 10}</t>
+          <t>{'east': -1.185206456727828, 'south': 52.54100635124824, 'north': 52.55899364875175, 'west': -1.214793543272172, 'accuracyLevel': 1}</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>['deployment']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -4008,22 +4008,22 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>lotus</t>
+          <t>electricbrands</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Leicestershire</t>
+          <t>Lower Saxony</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>{'east': -1.185206456727828, 'south': 52.54100635124824, 'north': 52.55899364875175, 'west': -1.214793543272172, 'accuracyLevel': 1}</t>
+          <t>{'east': 9.979687279962073, 'south': 51.505687276390006, 'north': 51.577160792979065, 'west': 9.878951301731295, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>electricbrands</t>
+          <t>gotion high tech</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4061,17 +4061,17 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>{'east': 9.979687279962073, 'south': 51.505687276390006, 'north': 51.577160792979065, 'west': 9.878951301731295, 'accuracyLevel': 10}</t>
+          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['cell' 'module_pack']</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>gotion high tech</t>
+          <t>graphenix development inc</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
+          <t>{'east': 9.39737487771509, 'south': 51.65144861839693, 'north': 51.66817163652086, 'west': 9.378799354242966, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>graphenix development inc</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>{'east': 9.39737487771509, 'south': 51.65144861839693, 'north': 51.66817163652086, 'west': 9.378799354242966, 'accuracyLevel': 10}</t>
+          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell' nan 'eam']</t>
         </is>
       </c>
     </row>
@@ -4175,17 +4175,17 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
+          <t>{'east': 7.24054018331388, 'south': 53.333469404564674, 'north': 53.39082510126331, 'west': 7.141750044104904, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>['cell' nan 'eam']</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>volkswagen group components</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4213,17 +4213,17 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>{'east': 7.24054018331388, 'south': 53.333469404564674, 'north': 53.39082510126331, 'west': 7.141750044104904, 'accuracyLevel': 10}</t>
+          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>volkswagen group components</t>
+          <t>volkswagen northvolt</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -4274,22 +4274,22 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>volkswagen northvolt</t>
+          <t>lg chem</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Lower Saxony</t>
+          <t>Lower Silesia</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>{'east': 10.45533584814119, 'south': 52.12864174128801, 'north': 52.19638022714064, 'west': 10.371113225395026, 'accuracyLevel': 10}</t>
+          <t>{'east': 16.942223164653207, 'south': 50.966038519670285, 'north': 50.97503216842171, 'west': 16.927939799213995, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>lg chem</t>
+          <t>lg energy solution</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>{'east': 16.942223164653207, 'south': 50.966038519670285, 'north': 50.97503216842171, 'west': 16.927939799213995, 'accuracyLevel': 2}</t>
+          <t>{'east': 17.19840487079657, 'south': 50.99657303935859, 'north': 51.203426960641416, 'west': 16.86826112920343, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -4350,22 +4350,22 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>lg energy solution</t>
+          <t>automotive cell company</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Lower Silesia</t>
+          <t>Molise</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>{'east': 17.19840487079657, 'south': 50.99657303935859, 'north': 51.203426960641416, 'west': 16.86826112920343, 'accuracyLevel': 2}</t>
+          <t>{'east': 15.02515803802899, 'south': 41.96664218357598, 'north': 42.006732149173125, 'west': 14.964670874620774, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -4388,22 +4388,22 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>automotive cell company</t>
+          <t>gotion inobat batteries</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Molise</t>
+          <t>Nitra Region</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>{'east': 15.02515803802899, 'south': 41.96664218357598, 'north': 42.006732149173125, 'west': 14.964670874620774, 'accuracyLevel': 10}</t>
+          <t>{'east': 18.203510679385108, 'south': 48.073414059960506, 'north': 48.09885194003949, 'west': 18.165421320614893, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -4426,22 +4426,22 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>gotion inobat batteries</t>
+          <t>freyr</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Nitra Region</t>
+          <t>Nordland</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>{'east': 18.203510679385108, 'south': 48.073414059960506, 'north': 48.09885194003949, 'west': 18.165421320614893, 'accuracyLevel': 2}</t>
+          <t>{'east': 15.533365159661637, 'south': 66.09555949009953, 'north': 66.78387692349938, 'west': 13.188270357919233, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['cell' 'eam']</t>
         </is>
       </c>
     </row>
@@ -4464,32 +4464,32 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>freyr</t>
+          <t>hopium</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Nordland</t>
+          <t>Normandy</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>{'east': 15.533365159661637, 'south': 66.09555949009953, 'north': 66.78387692349938, 'west': 13.188270357919233, 'accuracyLevel': 10}</t>
+          <t>{'east': 1.4948061634798788, 'south': 49.07231096191137, 'north': 49.113525038088625, 'west': 1.4318418365201213, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>['cell' 'eam']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>hopium</t>
+          <t>renault</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>{'east': 1.4948061634798788, 'south': 49.07231096191137, 'north': 49.113525038088625, 'west': 1.4318418365201213, 'accuracyLevel': 2}</t>
+          <t>{'east': 0.31886377737636096, 'south': 49.496896635124855, 'north': 49.49869536487515, 'west': 0.31609422262363907, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -4540,32 +4540,32 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>renault</t>
+          <t>cylib</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Normandy</t>
+          <t>North Rhine-Westphalia</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>{'east': 0.31886377737636096, 'south': 49.496896635124855, 'north': 49.49869536487515, 'west': 0.31609422262363907, 'accuracyLevel': 2}</t>
+          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>cylib</t>
+          <t>ego mobile</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4598,12 +4598,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ego mobile</t>
+          <t>ford</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
+          <t>{'east': 6.972890903720807, 'south': 50.915449013912095, 'north': 50.959219025077154, 'west': 6.927985101565835, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ford</t>
+          <t>fraunhofer ffb</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -4669,17 +4669,17 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>{'east': 6.972890903720807, 'south': 50.915449013912095, 'north': 50.959219025077154, 'west': 6.927985101565835, 'accuracyLevel': 10}</t>
+          <t>{'east': 7.671209105910431, 'south': 51.91537136540322, 'north': 51.98867213131061, 'west': 7.5839371596321765, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>fraunhofer ffb</t>
+          <t>nextego mobile</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -4707,17 +4707,17 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>{'east': 7.671209105910431, 'south': 51.91537136540322, 'north': 51.98867213131061, 'west': 7.5839371596321765, 'accuracyLevel': 10}</t>
+          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>nextego mobile</t>
+          <t>primobius</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4745,17 +4745,17 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
+          <t>{'east': 8.129861195726217, 'south': 50.98693272272397, 'north': 51.005533364701684, 'west': 8.079254137532761, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>primobius</t>
+          <t>pure battery technologies</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>{'east': 8.129861195726217, 'south': 50.98693272272397, 'north': 51.005533364701684, 'west': 8.079254137532761, 'accuracyLevel': 10}</t>
+          <t>{'east': 7.522725596119567, 'south': 51.34688986944242, 'north': 51.38640297699042, 'west': 7.436713019019417, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>pure battery technologies</t>
+          <t>rwth aachen university</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4821,7 +4821,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>{'east': 7.522725596119567, 'south': 51.34688986944242, 'north': 51.38640297699042, 'west': 7.436713019019417, 'accuracyLevel': 10}</t>
+          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -4844,22 +4844,22 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>rwth aachen university</t>
+          <t>britishvolt</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>North Rhine-Westphalia</t>
+          <t>Northumberland</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>{'east': 6.1438548677283755, 'south': 50.73892691283202, 'north': 50.80078678989726, 'west': 6.047295847418284, 'accuracyLevel': 10}</t>
+          <t>{'east': -1.486521581294416, 'south': 55.101808476974824, 'north': 55.148760091061156, 'west': -1.567174610804679, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>[nan 'cell' 'module_pack']</t>
         </is>
       </c>
     </row>
@@ -4882,22 +4882,22 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>britishvolt</t>
+          <t>forsee power</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Northumberland</t>
+          <t>Nouvelle-Aquitaine</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>{'east': -1.486521581294416, 'south': 55.101808476974824, 'north': 55.148760091061156, 'west': -1.567174610804679, 'accuracyLevel': 10}</t>
+          <t>{'east': 0.39865002888651413, 'south': 46.54472008430518, 'north': 46.62050191569482, 'west': 0.2883139711134859, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>[nan 'cell' 'module_pack']</t>
+          <t>['module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>forsee power</t>
+          <t>startec energy</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>{'east': 0.39865002888651413, 'south': 46.54472008430518, 'north': 46.62050191569482, 'west': 0.2883139711134859, 'accuracyLevel': 2}</t>
+          <t>{'east': -0.42813963484333717, 'south': 44.84478552998026, 'north': 44.85750447001975, 'west': -0.4460823651566629, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>['module_pack' nan]</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -4958,32 +4958,32 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>startec energy</t>
+          <t>revoz</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Novo Mesto</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>{'east': -0.42813963484333717, 'south': 44.84478552998026, 'north': 44.85750447001975, 'west': -0.4460823651566629, 'accuracyLevel': 2}</t>
+          <t>{'east': 15.211923613302544, 'south': 45.76816350041924, 'north': 45.84600721181288, 'west': 15.125180545809764, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -4996,32 +4996,32 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>revoz</t>
+          <t>ox2</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Novo Mesto</t>
+          <t>Opole Voivodeship</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>{'east': 15.211923613302544, 'south': 45.76816350041924, 'north': 45.84600721181288, 'west': 15.125180545809764, 'accuracyLevel': 10}</t>
+          <t>{'east': 17.635182972509067, 'south': 50.63194886119511, 'north': 50.652059271169065, 'west': 17.603464488428433, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['deployment']</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ox2</t>
+          <t>umicore</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -5049,17 +5049,17 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>{'east': 17.635182972509067, 'south': 50.63194886119511, 'north': 50.652059271169065, 'west': 17.603464488428433, 'accuracyLevel': 2}</t>
+          <t>{'east': 17.378517288819175, 'south': 50.44570251161992, 'north': 50.501867830070886, 'west': 17.290214400634028, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>['deployment']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -5072,22 +5072,22 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>umicore</t>
+          <t>finnish minerals group epsilon advanced materials</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Opole Voivodeship</t>
+          <t>Ostrobothnia</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>{'east': 17.378517288819175, 'south': 50.44570251161992, 'north': 50.501867830070886, 'west': 17.290214400634028, 'accuracyLevel': 2}</t>
+          <t>{'east': 21.69022613548251, 'south': 63.06235015650488, 'north': 63.12965246107453, 'west': 21.541318359146487, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>finnish minerals group epsilon advanced materials</t>
+          <t>freyr battery</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>freyr battery</t>
+          <t>johnson matthey</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5186,32 +5186,32 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>johnson matthey</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ostrobothnia</t>
+          <t>Oxfordshire</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>{'east': 21.69022613548251, 'south': 63.06235015650488, 'north': 63.12965246107453, 'west': 21.541318359146487, 'accuracyLevel': 2}</t>
+          <t>{'east': -1.177081863538468, 'south': 51.710079613642115, 'north': 51.796840007641904, 'west': -1.319509894915436, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>photovolt development partners</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -5239,17 +5239,17 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>{'east': -1.177081863538468, 'south': 51.710079613642115, 'north': 51.796840007641904, 'west': -1.319509894915436, 'accuracyLevel': 10}</t>
+          <t>{'east': -0.8700660028834721, 'south': 51.459409373196955, 'north': 52.16846751466819, 'west': -1.7195007584303506, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['deployment']</t>
         </is>
       </c>
     </row>
@@ -5262,32 +5262,32 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>photovolt development partners</t>
+          <t>samsung sdi</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Oxfordshire</t>
+          <t>Pest County</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>{'east': -0.8700660028834721, 'south': 51.459409373196955, 'north': 52.16846751466819, 'west': -1.7195007584303506, 'accuracyLevel': 10}</t>
+          <t>{'east': 19.158261729415546, 'south': 47.66702746913661, 'north': 47.69945453086339, 'west': 19.11008027058445, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>['deployment']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -5300,32 +5300,32 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>samsung sdi</t>
+          <t>fiat chrysler</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Pest County</t>
+          <t>Piedmont</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>{'east': 19.158261729415546, 'south': 47.66702746913661, 'north': 47.69945453086339, 'west': 19.11008027058445, 'accuracyLevel': 2}</t>
+          <t>{'east': 7.762857702337489, 'south': 45.00679706738262, 'north': 45.13352365046831, 'west': 7.5778599181360695, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>fiat chrysler</t>
+          <t>italvolt</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5353,17 +5353,17 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>{'east': 7.762857702337489, 'south': 45.00679706738262, 'north': 45.13352365046831, 'west': 7.5778599181360695, 'accuracyLevel': 10}</t>
+          <t>{'east': 7.844896013549455, 'south': 45.38066742905088, 'north': 45.388755825588596, 'west': 7.836848508602034, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>italvolt</t>
+          <t>micro mobility</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -5391,17 +5391,17 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>{'east': 7.844896013549455, 'south': 45.38066742905088, 'north': 45.388755825588596, 'west': 7.836848508602034, 'accuracyLevel': 10}</t>
+          <t>{'east': 7.762857702337489, 'south': 45.00679706738262, 'north': 45.13352365046831, 'west': 7.5778599181360695, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>micro mobility</t>
+          <t>stellantis</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -5452,32 +5452,32 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>stellantis</t>
+          <t>fortum</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Piedmont</t>
+          <t>Pirkanmaa</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>{'east': 7.762857702337489, 'south': 45.00679706738262, 'north': 45.13352365046831, 'west': 7.5778599181360695, 'accuracyLevel': 10}</t>
+          <t>{'east': 23.089090641514456, 'south': 61.758494786671086, 'north': 61.7805246370387, 'west': 23.042501155360544, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>fortum</t>
+          <t>fortum battery recycling</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -5528,22 +5528,22 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>fortum battery recycling</t>
+          <t>northvolt south bay solutions</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Pirkanmaa</t>
+          <t>Pomerania</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>{'east': 23.089090641514456, 'south': 61.758494786671086, 'north': 61.7805246370387, 'west': 23.042501155360544, 'accuracyLevel': 2}</t>
+          <t>{'east': 18.800645169287666, 'south': 54.26415059853274, 'north': 54.44038940146726, 'west': 18.497594830712334, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -5566,22 +5566,22 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>northvolt south bay solutions</t>
+          <t>automotive cell company</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Pomerania</t>
+          <t>Rheinland-Pfalz</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>{'east': 18.800645169287666, 'south': 54.26415059853274, 'north': 54.44038940146726, 'west': 18.497594830712334, 'accuracyLevel': 2}</t>
+          <t>{'east': 7.846920817292972, 'south': 49.41912208001153, 'north': 49.45860979846688, 'west': 7.6563392399020875, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['cell' 'module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>automotive cell company</t>
+          <t>e lyte</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack' nan]</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -5642,32 +5642,32 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>e lyte</t>
+          <t>sng solar</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Rheinland-Pfalz</t>
+          <t>Riga</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>{'east': 7.846920817292972, 'south': 49.41912208001153, 'north': 49.45860979846688, 'west': 7.6563392399020875, 'accuracyLevel': 10}</t>
+          <t>{'east': 24.311465500035062, 'south': 56.83421483411752, 'north': 57.05779339669368, 'west': 23.900318862757935, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['deployment']</t>
         </is>
       </c>
     </row>
@@ -5680,32 +5680,32 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>sng solar</t>
+          <t>eberspacher</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>BG</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Riga</t>
+          <t>Ruse</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>{'east': 24.311465500035062, 'south': 56.83421483411752, 'north': 57.05779339669368, 'west': 23.900318862757935, 'accuracyLevel': 2}</t>
+          <t>{'east': 26.46456200000006, 'south': 43.314156000000054, 'north': 44.03866720000011, 'west': 25.45826200000009, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>['deployment']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -5718,32 +5718,32 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>eberspacher</t>
+          <t>svolt</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>BG</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Ruse</t>
+          <t>Saarland</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>{'east': 26.46456200000006, 'south': 43.314156000000054, 'north': 44.03866720000011, 'west': 25.45826200000009, 'accuracyLevel': 10}</t>
+          <t>{'east': 6.712134539665601, 'south': 49.23040732223842, 'north': 49.248954527013105, 'west': 6.689386163775832, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -5756,22 +5756,22 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>svolt</t>
+          <t>li cycle glencore</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Saarland</t>
+          <t>Sardinia</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>{'east': 6.712134539665601, 'south': 49.23040732223842, 'north': 49.248954527013105, 'west': 6.689386163775832, 'accuracyLevel': 10}</t>
+          <t>{'east': 9.82842015716897, 'south': 38.8591910527341, 'north': 41.3133205526259, 'west': 8.13072799347893, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -5794,22 +5794,22 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>li cycle glencore</t>
+          <t>basf</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Sardinia</t>
+          <t>Satakunta</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>{'east': 9.82842015716897, 'south': 38.8591910527341, 'north': 41.3133205526259, 'west': 8.13072799347893, 'accuracyLevel': 10}</t>
+          <t>{'east': 22.15629064481865, 'south': 61.30565177481619, 'north': 61.32768162518381, 'west': 22.11037595518135, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -5832,22 +5832,22 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>basf</t>
+          <t>blackstone technology</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Satakunta</t>
+          <t>Saxony</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>{'east': 22.15629064481865, 'south': 61.30565177481619, 'north': 61.32768162518381, 'west': 22.11037595518135, 'accuracyLevel': 2}</t>
+          <t>{'east': 13.170802679046409, 'south': 51.11103302752995, 'north': 51.142678785040744, 'west': 13.087836468078457, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>blackstone technology</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>{'east': 13.170802679046409, 'south': 51.11103302752995, 'north': 51.142678785040744, 'west': 13.087836468078457, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.411756004510003, 'south': 51.31210421575785, 'north': 51.35997944123762, 'west': 12.347875462041682, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -5895,7 +5895,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -5928,12 +5928,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>[nan 'electric']</t>
         </is>
       </c>
     </row>
@@ -5946,7 +5946,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>european semiconductor manufacturing company</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -5961,17 +5961,17 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>{'east': 12.411756004510003, 'south': 51.31210421575785, 'north': 51.35997944123762, 'west': 12.347875462041682, 'accuracyLevel': 10}</t>
+          <t>{'east': 13.786581145811093, 'south': 51.027883739261306, 'north': 51.07425076373171, 'west': 13.688065285884342, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>[nan 'electric']</t>
+          <t>['ingot_wafer']</t>
         </is>
       </c>
     </row>
@@ -5984,7 +5984,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>european semiconductor manufacturing company</t>
+          <t>jt energy systems</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -5999,17 +5999,17 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>{'east': 13.786581145811093, 'south': 51.027883739261306, 'north': 51.07425076373171, 'west': 13.688065285884342, 'accuracyLevel': 10}</t>
+          <t>{'east': 13.377158995430786, 'south': 50.89650634923862, 'north': 50.93969230494892, 'west': 13.311327599881487, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>['ingot_wafer']</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>jt energy systems</t>
+          <t>meyer burger</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -6037,17 +6037,17 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>{'east': 13.377158995430786, 'south': 50.89650634923862, 'north': 50.93969230494892, 'west': 13.311327599881487, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.86416539007656, 'south': 50.69177535124857, 'north': 50.70976264875143, 'west': 12.835760609923442, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>meyer burger</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -6075,17 +6075,17 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>{'east': 12.86416539007656, 'south': 50.69177535124857, 'north': 50.70976264875143, 'west': 12.835760609923442, 'accuracyLevel': 2}</t>
+          <t>{'east': 12.550681217373935, 'south': 50.69208436668295, 'north': 50.7538028554246, 'west': 12.431212728003908, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>[nan 'electric']</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>porsche</t>
+          <t>amg lithium</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -6108,12 +6108,12 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Saxony</t>
+          <t>Saxony-Anhalt</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>{'east': 12.411756004510003, 'south': 51.31210421575785, 'north': 51.35997944123762, 'west': 12.347875462041682, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.351755668282912, 'south': 51.6050106188674, 'north': 51.64429590459737, 'west': 12.282901278442232, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>battery lifecycle company</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -6146,22 +6146,22 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Saxony</t>
+          <t>Saxony-Anhalt</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>{'east': 12.550681217373935, 'south': 50.69208436668295, 'north': 50.7538028554246, 'west': 12.431212728003908, 'accuracyLevel': 10}</t>
+          <t>{'east': 11.666155627612763, 'south': 52.11302392312941, 'north': 52.16994742032871, 'west': 11.572401049348347, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>[nan 'electric']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -6174,7 +6174,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>amg lithium</t>
+          <t>farasis energy</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6212,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>battery lifecycle company</t>
+          <t>farasis energy europe</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>{'east': 11.666155627612763, 'south': 52.11302392312941, 'north': 52.16994742032871, 'west': 11.572401049348347, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.351755668282912, 'south': 51.6050106188674, 'north': 51.64429590459737, 'west': 12.282901278442232, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6250,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>farasis energy</t>
+          <t>li cycle</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>{'east': 12.351755668282912, 'south': 51.6050106188674, 'north': 51.64429590459737, 'west': 12.282901278442232, 'accuracyLevel': 10}</t>
+          <t>{'east': 11.666155627612763, 'south': 52.11302392312941, 'north': 52.16994742032871, 'west': 11.572401049348347, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>farasis energy europe</t>
+          <t>norcsi</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>{'east': 12.351755668282912, 'south': 51.6050106188674, 'north': 51.64429590459737, 'west': 12.282901278442232, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.007894073905979, 'south': 51.46824374507202, 'north': 51.4972081039573, 'west': 11.955331565791347, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>li cycle</t>
+          <t>northvolt</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -6336,12 +6336,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Saxony-Anhalt</t>
+          <t>Schleswig-Holstein</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>{'east': 11.666155627612763, 'south': 52.11302392312941, 'north': 52.16994742032871, 'west': 11.572401049348347, 'accuracyLevel': 10}</t>
+          <t>{'east': 9.138809415376675, 'south': 54.17658006003535, 'north': 54.21275817621844, 'west': 9.072678883413348, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -6364,22 +6364,22 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>norcsi</t>
+          <t>ecovolta</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Saxony-Anhalt</t>
+          <t>Schwyz</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>{'east': 12.007894073905979, 'south': 51.46824374507202, 'north': 51.4972081039573, 'west': 11.955331565791347, 'accuracyLevel': 10}</t>
+          <t>{'east': 8.665515373442128, 'south': 47.014318672227304, 'north': 47.03028574910165, 'west': 8.63886730772937, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -6402,22 +6402,22 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>northvolt</t>
+          <t>calb</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Schleswig-Holstein</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>{'east': 9.138809415376675, 'south': 54.17658006003535, 'north': 54.21275817621844, 'west': 9.072678883413348, 'accuracyLevel': 10}</t>
+          <t>{'east': -8.681435537087584, 'south': 37.865777084375594, 'north': 38.04929489872405, 'west': -8.890550901882476, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>['cell' 'module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -6440,27 +6440,27 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>ecovolta</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Schwyz</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>{'east': 8.665515373442128, 'south': 47.014318672227304, 'north': 47.03028574910165, 'west': 8.63886730772937, 'accuracyLevel': 10}</t>
+          <t>{'east': -8.879729959021228, 'south': 38.55219542385758, 'north': 38.585846576142416, 'west': -8.922780040978774, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -6478,22 +6478,22 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>calb</t>
+          <t>ae elemental</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Silesia</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>{'east': -8.681435537087584, 'south': 37.865777084375594, 'north': 38.04929489872405, 'west': -8.890550901882476, 'accuracyLevel': 10}</t>
+          <t>{'east': 19.46370186425747, 'south': 50.45782940973647, 'north': 50.51748652654593, 'west': 19.36987815283233, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack' nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -6516,22 +6516,22 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>stellantis</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Silesia</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>{'east': -8.879729959021228, 'south': 38.55219542385758, 'north': 38.585846576142416, 'west': -8.922780040978774, 'accuracyLevel': 2}</t>
+          <t>{'east': 19.03939220706789, 'south': 50.090434630251295, 'north': 50.1838993697487, 'west': 18.89342779293211, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -6554,22 +6554,22 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>ae elemental</t>
+          <t>librec</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Silesia</t>
+          <t>Solothurn</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>{'east': 19.46370186425747, 'south': 50.45782940973647, 'north': 50.51748652654593, 'west': 19.36987815283233, 'accuracyLevel': 2}</t>
+          <t>{'east': 7.576800610512958, 'south': 47.17046994348771, 'north': 47.19454268087654, 'west': 7.54760484225659, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -6592,32 +6592,32 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>stellantis</t>
+          <t>agratas</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Silesia</t>
+          <t>Somerset</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>{'east': 19.03939220706789, 'south': 50.090434630251295, 'north': 50.1838993697487, 'west': 18.89342779293211, 'accuracyLevel': 2}</t>
+          <t>{'east': -2.966574158866892, 'south': 51.09991785910348, 'north': 51.16072612199926, 'west': -3.040637001994926, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -6630,22 +6630,22 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>librec</t>
+          <t>valmet automotive</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Solothurn</t>
+          <t>Southwest Finland</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>{'east': 7.576800610512958, 'south': 47.17046994348771, 'north': 47.19454268087654, 'west': 7.54760484225659, 'accuracyLevel': 10}</t>
+          <t>{'east': 23.17405173521075, 'south': 60.36322289002605, 'north': 60.40344370997394, 'west': 23.09261486478925, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -6655,7 +6655,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -6668,32 +6668,32 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>agratas</t>
+          <t>valmet automotive</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Somerset</t>
+          <t>Southwest Finland</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>{'east': -2.966574158866892, 'south': 51.09991785910348, 'north': 51.16072612199926, 'west': -3.040637001994926, 'accuracyLevel': 10}</t>
+          <t>{'east': 21.44165659811968, 'south': 60.78421721753881, 'north': 60.81664427926559, 'west': 21.37515400979052, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -6706,32 +6706,32 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>valmet automotive</t>
+          <t>tesla</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Southwest Finland</t>
+          <t>State of Berlin</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>{'east': 23.17405173521075, 'south': 60.36322289002605, 'north': 60.40344370997394, 'west': 23.09261486478925, 'accuracyLevel': 2}</t>
+          <t>{'east': 13.7604692835498, 'south': 52.3382418348765, 'north': 52.6749171487584, 'west': 13.0883332178678, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['electric']</t>
         </is>
       </c>
     </row>
@@ -6744,32 +6744,32 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>valmet automotive</t>
+          <t>aesc</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Southwest Finland</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>{'east': 21.44165659811968, 'south': 60.78421721753881, 'north': 60.81664427926559, 'west': 21.37515400979052, 'accuracyLevel': 2}</t>
+          <t>{'east': -1.351172911278187, 'south': 54.85601261436129, 'north': 54.939914387340465, 'west': -1.480882124121284, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['cell' 'module_pack' nan]</t>
         </is>
       </c>
     </row>
@@ -6782,32 +6782,32 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>tesla</t>
+          <t>nissan</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>State of Berlin</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>{'east': 13.7604692835498, 'south': 52.3382418348765, 'north': 52.6749171487584, 'west': 13.0883332178678, 'accuracyLevel': 10}</t>
+          <t>{'east': -1.351172911278187, 'south': 54.85601261436129, 'north': 54.939914387340465, 'west': -1.480882124121284, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>['electric']</t>
+          <t>['cell' nan]</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>aesc</t>
+          <t>nissan</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -6840,12 +6840,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack' nan]</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -6858,7 +6858,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>nissan</t>
+          <t>saietta group</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>['cell' nan]</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -6896,32 +6896,32 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>nissan</t>
+          <t>vianode</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Telemark</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>{'east': -1.351172911278187, 'south': 54.85601261436129, 'north': 54.939914387340465, 'west': -1.480882124121284, 'accuracyLevel': 10}</t>
+          <t>{'east': 9.650593931856756, 'south': 59.11056163512485, 'north': 59.112360364875144, 'west': 9.647090068143244, 'accuracyLevel': 1}</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>['eam']</t>
         </is>
       </c>
     </row>
@@ -6934,32 +6934,32 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>saietta group</t>
+          <t>catl</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Thuringia</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>{'east': -1.351172911278187, 'south': 54.85601261436129, 'north': 54.939914387340465, 'west': -1.480882124121284, 'accuracyLevel': 10}</t>
+          <t>{'east': 11.042818518511504, 'south': 50.96796336832227, 'north': 50.98661954344408, 'west': 11.012904147220443, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>[nan 'cell']</t>
         </is>
       </c>
     </row>
@@ -6972,22 +6972,22 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>vianode</t>
+          <t>lion smart</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Telemark</t>
+          <t>Thuringia</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>{'east': 9.650593931856756, 'south': 59.11056163512485, 'north': 59.112360364875144, 'west': 9.647090068143244, 'accuracyLevel': 1}</t>
+          <t>{'east': 10.75616528468898, 'south': 50.4175597443067, 'north': 50.43717896182797, 'west': 10.710515273546633, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>['eam']</t>
+          <t>['module_pack']</t>
         </is>
       </c>
     </row>
@@ -7010,7 +7010,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>catl</t>
+          <t>sungeel hitech and samsung</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -7025,7 +7025,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>{'east': 11.042818518511504, 'south': 50.96796336832227, 'north': 50.98661954344408, 'west': 11.012904147220443, 'accuracyLevel': 10}</t>
+          <t>{'east': 12.1244000937386, 'south': 50.82512988478043, 'north': 50.9200134673793, 'west': 12.043412258178638, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>[nan 'cell']</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -7048,22 +7048,22 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>lion smart</t>
+          <t>gotion inobat batteries</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Thuringia</t>
+          <t>Trnava Region</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>{'east': 10.75616528468898, 'south': 50.4175597443067, 'north': 50.43717896182797, 'west': 10.710515273546633, 'accuracyLevel': 10}</t>
+          <t>{'east': 17.566157352814365, 'south': 48.27251017562412, 'north': 48.281503824375875, 'west': 17.552642647185635, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -7073,7 +7073,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>['module_pack']</t>
+          <t>['cell']</t>
         </is>
       </c>
     </row>
@@ -7086,22 +7086,22 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>sungeel hitech and samsung</t>
+          <t>inobat</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Thuringia</t>
+          <t>Trnava Region</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>{'east': 12.1244000937386, 'south': 50.82512988478043, 'north': 50.9200134673793, 'west': 12.043412258178638, 'accuracyLevel': 10}</t>
+          <t>{'east': 17.566157352814365, 'south': 48.27251017562412, 'north': 48.281503824375875, 'west': 17.552642647185635, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>['recycling']</t>
+          <t>['cell' 'module_pack']</t>
         </is>
       </c>
     </row>
@@ -7124,22 +7124,22 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>gotion inobat batteries</t>
+          <t>elinor batteries</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Trnava Region</t>
+          <t>Trøndelag</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>{'east': 17.566157352814365, 'south': 48.27251017562412, 'north': 48.281503824375875, 'west': 17.552642647185635, 'accuracyLevel': 2}</t>
+          <t>{'east': 10.0138512334075, 'south': 62.8904313423315, 'north': 63.6465504546332, 'west': 9.17706499974905, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -7162,32 +7162,32 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>inobat</t>
+          <t>ignitis renewables</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Trnava Region</t>
+          <t>Tukums Municipality</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>{'east': 17.566157352814365, 'south': 48.27251017562412, 'north': 48.281503824375875, 'west': 17.552642647185635, 'accuracyLevel': 2}</t>
+          <t>{'east': 23.10391894070486, 'south': 56.92760035124857, 'north': 56.94558764875143, 'west': 23.07094105929514, 'accuracyLevel': 1}</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>['cell' 'module_pack']</t>
+          <t>['deployment']</t>
         </is>
       </c>
     </row>
@@ -7200,32 +7200,32 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>elinor batteries</t>
+          <t>european energy</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Trøndelag</t>
+          <t>Utena</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>{'east': 10.0138512334075, 'south': 62.8904313423315, 'north': 63.6465504546332, 'west': 9.17706499974905, 'accuracyLevel': 10}</t>
+          <t>{'east': 25.12512133757019, 'south': 55.5128509433159, 'north': 55.53828882339488, 'west': 25.08016659577942, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>solar</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>['cell']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -7238,32 +7238,32 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ignitis renewables</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Tukums Municipality</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>{'east': 23.10391894070486, 'south': 56.92760035124857, 'north': 56.94558764875143, 'west': 23.07094105929514, 'accuracyLevel': 1}</t>
+          <t>{'east': -0.2233115815890593, 'south': 39.6499839578681, 'north': 39.7166826421319, 'west': -0.3100218184109407, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>['deployment']</t>
+          <t>['cell' nan 'eam']</t>
         </is>
       </c>
     </row>
@@ -7276,32 +7276,32 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>european energy</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Utena</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>{'east': 25.12512133757019, 'south': 55.5128509433159, 'north': 55.53828882339488, 'west': 25.08016659577942, 'accuracyLevel': 2}</t>
+          <t>{'east': -0.2233115815890593, 'south': 39.6499839578681, 'north': 39.7166826421319, 'west': -0.3100218184109407, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>solar</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>[nan 'electric']</t>
         </is>
       </c>
     </row>
@@ -7314,32 +7314,32 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>schaeffler</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Vas County</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>{'east': -0.2233115815890593, 'south': 39.6499839578681, 'north': 39.7166826421319, 'west': -0.3100218184109407, 'accuracyLevel': 2}</t>
+          <t>{'east': 16.67497971157691, 'south': 47.19462165724717, 'north': 47.267130771578834, 'west': 16.568125699952688, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>vehicle</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>['cell' nan 'eam']</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -7352,22 +7352,22 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>stellantis</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Viseu</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>{'east': -0.2233115815890593, 'south': 39.6499839578681, 'north': 39.7166826421319, 'west': -0.3100218184109407, 'accuracyLevel': 2}</t>
+          <t>{'east': -7.745476611297256, 'south': 40.59235052101233, 'north': 40.61614547898767, 'west': -7.776823388702743, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -7390,22 +7390,22 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>schaeffler</t>
+          <t>london taxi company</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Vas County</t>
+          <t>Warwickshire</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>{'east': 16.67497971157691, 'south': 47.19462165724717, 'north': 47.267130771578834, 'west': 16.568125699952688, 'accuracyLevel': 2}</t>
+          <t>{'east': -1.4019123625614562, 'south': 52.42433965124857, 'north': 52.44232694875143, 'west': -1.4314210374385437, 'accuracyLevel': 1}</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -7415,7 +7415,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['electric' nan]</t>
         </is>
       </c>
     </row>
@@ -7428,32 +7428,32 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>stellantis</t>
+          <t>recyclus group</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Viseu</t>
+          <t>Wolverhampton</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>{'east': -7.745476611297256, 'south': 40.59235052101233, 'north': 40.61614547898767, 'west': -7.776823388702743, 'accuracyLevel': 2}</t>
+          <t>{'east': -2.047589062994391, 'south': 52.543274219952295, 'north': 52.64243985317021, 'west': -2.208067813103782, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>[nan 'electric']</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -7466,32 +7466,32 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>london taxi company</t>
+          <t>battrion</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Warwickshire</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>{'east': -1.4019123625614562, 'south': 52.42433965124857, 'north': 52.44232694875143, 'west': -1.4314210374385437, 'accuracyLevel': 1}</t>
+          <t>{'east': 8.651844002323093, 'south': 47.38425215646728, 'north': 47.408586863663956, 'west': 8.589968123394014, 'accuracyLevel': 10}</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>vehicle</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>['electric' nan]</t>
+          <t>[nan]</t>
         </is>
       </c>
     </row>
@@ -7504,22 +7504,22 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>recyclus group</t>
+          <t>lg energy solution derichebourg</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Wolverhampton</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>{'east': -2.047589062994391, 'south': 52.543274219952295, 'north': 52.64243985317021, 'west': -2.208067813103782, 'accuracyLevel': 10}</t>
+          <t>{'east': 2.3376845881749038, 'south': 49.14977227170855, 'north': 49.16534972829145, 'west': 2.313861411825096, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -7542,22 +7542,22 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>battrion</t>
+          <t>hydrovolt</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Østfold</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>{'east': 8.651844002323093, 'south': 47.38425215646728, 'north': 47.408586863663956, 'west': 8.589968123394014, 'accuracyLevel': 10}</t>
+          <t>{'east': 11.002868481159044, 'south': 59.180746571333344, 'north': 59.255453428666655, 'west': 10.856731518840956, 'accuracyLevel': 2}</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -7567,7 +7567,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>[nan]</t>
+          <t>['recycling']</t>
         </is>
       </c>
     </row>
@@ -7580,22 +7580,22 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>lg energy solution derichebourg</t>
+          <t>green cell</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Świętokrzyskie</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>{'east': 2.3376845881749038, 'south': 49.14977227170855, 'north': 49.16534972829145, 'west': 2.313861411825096, 'accuracyLevel': 2}</t>
+          <t>{'east': 20.84852492504332, 'south': 50.5355329482598, 'north': 50.553520245762655, 'west': 20.820214393804335, 'accuracyLevel': 1}</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -7604,82 +7604,6 @@
         </is>
       </c>
       <c r="H189" t="inlineStr">
-        <is>
-          <t>['recycling']</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="1" t="n">
-        <v>188</v>
-      </c>
-      <c r="B190" t="n">
-        <v>189</v>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>hydrovolt</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Østfold</t>
-        </is>
-      </c>
-      <c r="F190" t="inlineStr">
-        <is>
-          <t>{'east': 11.002868481159044, 'south': 59.180746571333344, 'north': 59.255453428666655, 'west': 10.856731518840956, 'accuracyLevel': 2}</t>
-        </is>
-      </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>battery</t>
-        </is>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>['recycling']</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="1" t="n">
-        <v>189</v>
-      </c>
-      <c r="B191" t="n">
-        <v>190</v>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>green cell</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Świętokrzyskie</t>
-        </is>
-      </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>{'east': 20.84852492504332, 'south': 50.5355329482598, 'north': 50.553520245762655, 'west': 20.820214393804335, 'accuracyLevel': 1}</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>battery</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
         <is>
           <t>['module_pack']</t>
         </is>

</xml_diff>